<commit_message>
Add Google Ads actuals and EUR conversion to 2026 spend workbook
Google Ads monthly cost Jan-Sep 2026 (EUR) from the campaign report,
ChatGPT Ads moved to EUR, single EUR->USD rate input on the Summary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jw6zcgNAxCa88wNrGAsFKC
</commit_message>
<xml_diff>
--- a/PNP_Paid_Ads_Spend_2026.xlsx
+++ b/PNP_Paid_Ads_Spend_2026.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="94">
   <si>
     <t xml:space="preserve">Plug and Play – Paid Ads Spend 2026</t>
   </si>
@@ -31,10 +31,13 @@
     <t xml:space="preserve">Data up to:</t>
   </si>
   <si>
-    <t xml:space="preserve">Data status:  Meta ✔   ChatGPT ✔   Google ✘ (waiting for export)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Spend vs. budget by platform (USD)</t>
+    <t xml:space="preserve">EUR → USD rate used:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈ 2026 average so far. Replace with the rate Finance uses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Spend vs. budget by platform (all in USD)</t>
   </si>
   <si>
     <t xml:space="preserve">Platform</t>
@@ -71,7 +74,7 @@
     <t xml:space="preserve">Meta</t>
   </si>
   <si>
-    <t xml:space="preserve">Google</t>
+    <t xml:space="preserve">Google Ads</t>
   </si>
   <si>
     <t xml:space="preserve">Total Meta + Google ($270k budget)</t>
@@ -83,7 +86,7 @@
     <t xml:space="preserve">Grand total – all platforms</t>
   </si>
   <si>
-    <t xml:space="preserve">ChatGPT Ads is paid outside the $270k budget. Add its budget in B10 if it gets one.</t>
+    <t xml:space="preserve">Google Ads and ChatGPT Ads are billed in EUR and converted at the rate in B3. ChatGPT Ads is paid outside the $270k budget.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Key numbers</t>
@@ -107,19 +110,16 @@
     <t xml:space="preserve">Budget left for Oct–Dec if we stretch</t>
   </si>
   <si>
-    <t xml:space="preserve">Red % = 90% or more of the annual budget already spent.</t>
+    <t xml:space="preserve">Google Ads spent so far, in EUR (as billed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red = 90% or more of the annual budget already spent, or over budget.</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly Spend 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Yellow cells = type here. Blue numbers = taken from the platform exports. Black = calculated.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EUR → USD rate:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder – confirm the rate Finance uses. Put 1 if the Google account is actually in USD.</t>
+    <t xml:space="preserve">Amounts in the currency each platform bills in. Yellow cells = type here. The Total column converts everything to USD using the rate on the Summary tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Month</t>
@@ -132,22 +132,18 @@
 (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Google
-(EUR, as exported)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google
+    <t xml:space="preserve">Google Ads
+(EUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ChatGPT Ads
+(EUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total
 (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">ChatGPT Ads
-(USD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total all platforms
-(USD)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jan 2026</t>
   </si>
   <si>
@@ -199,13 +195,16 @@
     <t xml:space="preserve">TOTAL 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Meta: 'Plug and Play Tech Center – Dollars' ad account export, Amount spent (USD), 1 Jan – 30 Sep 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google: waiting for the export (Cost by month, 1 Jan – 30 Sep 2026).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ChatGPT Ads: 'Test 1' campaign, 23 Sep – 2 Oct 2026, total $229.56. Entered in September; the last ~2 days may belong to October.</t>
+    <t xml:space="preserve">Sources (exported 8 Oct 2026, period 1 Jan – 30 Sep 2026):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Meta: 'Plug and Play Tech Center – Dollars' ad account (the only active account), 'Amount spent (USD)'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Google Ads: Campaign report, 'Cost' (EUR), monthly account totals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ChatGPT Ads: 'Test 1' campaign, 23 Sep – 2 Oct 2026, €229.56 total. Put in September; the last ~2 days may belong to October.</t>
   </si>
   <si>
     <t xml:space="preserve">Spend by Territory – Jan to Sep 2026 (for reference only)</t>
@@ -217,6 +216,9 @@
     <t xml:space="preserve">Territory</t>
   </si>
   <si>
+    <t xml:space="preserve">Google</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total spent</t>
   </si>
   <si>
@@ -268,7 +270,7 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Red = over its territory budget. These territory budgets add up to $294,676, not $270,000, and its Meta total ($167,062) is lower than the Meta export ($178,067).</t>
+    <t xml:space="preserve">Red = over its territory budget. These territory budgets add up to $294,676, not $270,000, and its totals don't match the platform exports (Meta $167,062 vs $178,067; Google 82,856 vs €89,718).</t>
   </si>
   <si>
     <t xml:space="preserve">How to update this sheet</t>
@@ -280,10 +282,10 @@
     <t xml:space="preserve">2. Type each month's amount into the yellow cells on the 'Monthly Spend' tab.</t>
   </si>
   <si>
-    <t xml:space="preserve">   • Meta → 'Meta (USD)'   • Google → 'Google (EUR, as exported)' – it converts to USD by itself   • ChatGPT → 'ChatGPT Ads (USD)'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Change 'Data up to' on the Summary tab, and the data-status line next to it.</t>
+    <t xml:space="preserve">   • Meta → 'Meta (USD)'   • Google → 'Google Ads (EUR)'   • ChatGPT → 'ChatGPT Ads (EUR)'  – the sheet converts EUR to USD by itself</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Change 'Data up to' on the Summary tab (and the EUR → USD rate if Finance gives you a new one).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Everything else (quarters, totals, budget left) updates by itself.</t>
@@ -304,7 +306,7 @@
     <t xml:space="preserve">• Last quarter = Q3 2026 (July–September).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Meta account is billed in USD. Google account is billed in EUR → converted at the rate on 'Monthly Spend' (C3).</t>
+    <t xml:space="preserve">• Meta is billed in USD. Google Ads and ChatGPT Ads are billed in EUR → converted at the rate on the Summary tab (B3).</t>
   </si>
   <si>
     <t xml:space="preserve">• Spend = 'Amount spent' (Meta) / 'Cost' (Google) as reported by the platform, before tax.</t>
@@ -320,9 +322,9 @@
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mmm\ d&quot;, &quot;yyyy"/>
-    <numFmt numFmtId="166" formatCode="\$#,##0;&quot;-$&quot;#,##0;\-"/>
-    <numFmt numFmtId="167" formatCode="0%;\-0%;\-"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.00"/>
+    <numFmt numFmtId="167" formatCode="\$#,##0;&quot;-$&quot;#,##0;\-"/>
+    <numFmt numFmtId="168" formatCode="0%;\-0%;\-"/>
     <numFmt numFmtId="169" formatCode="\€#,##0;&quot;-€&quot;#,##0;\-"/>
   </numFmts>
   <fonts count="14">
@@ -505,7 +507,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -519,6 +521,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -538,23 +544,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -562,14 +568,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -578,11 +588,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -595,10 +605,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -873,7 +879,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -897,291 +903,313 @@
       <c r="B2" s="3" t="n">
         <v>46295</v>
       </c>
-      <c r="D2" s="4" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="B3" s="4" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="8" t="n">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="9" t="n">
         <v>180000</v>
       </c>
-      <c r="C6" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!C6:C8)</f>
+      <c r="C7" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!C5:C7)</f>
         <v>75432.1</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!C9:C11)</f>
+      <c r="D7" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!C8:C10)</f>
         <v>61971.35</v>
       </c>
-      <c r="E6" s="10" t="n">
-        <f aca="false">SUM('Monthly Spend'!C12:C14)</f>
+      <c r="E7" s="11" t="n">
+        <f aca="false">SUM('Monthly Spend'!C11:C13)</f>
         <v>40663.58</v>
       </c>
-      <c r="F6" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!C15:C17)</f>
+      <c r="F7" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!C14:C16)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="11" t="n">
-        <f aca="false">SUM(C6:F6)</f>
+      <c r="G7" s="12" t="n">
+        <f aca="false">SUM(C7:F7)</f>
         <v>178067.03</v>
       </c>
-      <c r="H6" s="9" t="n">
-        <f aca="false">IF(B6="","",B6-G6)</f>
+      <c r="H7" s="10" t="n">
+        <f aca="false">IF(B7="","",B7-G7)</f>
         <v>1932.96999999997</v>
       </c>
-      <c r="I6" s="12" t="n">
-        <f aca="false">IF(B6="","",G6/B6)</f>
+      <c r="I7" s="13" t="n">
+        <f aca="false">IF(B7="","",G7/B7)</f>
         <v>0.989261277777778</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="8" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="9" t="n">
         <v>90000</v>
       </c>
-      <c r="C7" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!E6:E8)</f>
+      <c r="C8" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!D5:D7)*Summary!$B$3</f>
+        <v>33248.906</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!D8:D10)*Summary!$B$3</f>
+        <v>37354.4244</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <f aca="false">SUM('Monthly Spend'!D11:D13)*Summary!$B$3</f>
+        <v>33469.4684</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!D14:D16)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!E9:E11)</f>
+      <c r="G8" s="12" t="n">
+        <f aca="false">SUM(C8:F8)</f>
+        <v>104072.7988</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <f aca="false">IF(B8="","",B8-G8)</f>
+        <v>-14072.7988</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <f aca="false">IF(B8="","",G8/B8)</f>
+        <v>1.15636443111111</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="15" t="n">
+        <f aca="false">SUM(B7:B8)</f>
+        <v>270000</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <f aca="false">SUM(C7:C8)</f>
+        <v>108681.006</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <f aca="false">SUM(D7:D8)</f>
+        <v>99325.7744</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <f aca="false">SUM(E7:E8)</f>
+        <v>74133.0484</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <f aca="false">SUM(F7:F8)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="10" t="n">
-        <f aca="false">SUM('Monthly Spend'!E12:E14)</f>
+      <c r="G9" s="15" t="n">
+        <f aca="false">SUM(G7:G8)</f>
+        <v>282139.8288</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <f aca="false">SUM(H7:H8)</f>
+        <v>-12139.8288</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <f aca="false">IF(B9=0,"",G9/B9)</f>
+        <v>1.04496232888889</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="17"/>
+      <c r="C11" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!E5:E7)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="F7" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!E15:E17)</f>
+      <c r="D11" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!E8:E10)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="G7" s="11" t="n">
-        <f aca="false">SUM(C7:F7)</f>
+      <c r="E11" s="11" t="n">
+        <f aca="false">SUM('Monthly Spend'!E11:E13)*Summary!$B$3</f>
+        <v>266.2896</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!E14:E16)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="H7" s="9" t="n">
-        <f aca="false">IF(B7="","",B7-G7)</f>
-        <v>90000</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <f aca="false">IF(B7="","",G7/B7)</f>
+      <c r="G11" s="12" t="n">
+        <f aca="false">SUM(C11:F11)</f>
+        <v>266.2896</v>
+      </c>
+      <c r="H11" s="10" t="str">
+        <f aca="false">IF(B11="","",B11-G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="13" t="str">
+        <f aca="false">IF(B11="","",G11/B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="15" t="n">
+        <f aca="false">C9+C11</f>
+        <v>108681.006</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <f aca="false">D9+D11</f>
+        <v>99325.7744</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <f aca="false">E9+E11</f>
+        <v>74399.338</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <f aca="false">F9+F11</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="14" t="n">
-        <f aca="false">SUM(B6:B7)</f>
+      <c r="G12" s="15" t="n">
+        <f aca="false">G9+G11</f>
+        <v>282406.1184</v>
+      </c>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="12" t="n">
+        <f aca="false">E12</f>
+        <v>74399.338</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="12" t="n">
+        <f aca="false">G12</f>
+        <v>282406.1184</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="12" t="n">
+        <f aca="false">B9</f>
         <v>270000</v>
       </c>
-      <c r="C8" s="14" t="n">
-        <f aca="false">SUM(C6:C7)</f>
-        <v>75432.1</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <f aca="false">SUM(D6:D7)</f>
-        <v>61971.35</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <f aca="false">SUM(E6:E7)</f>
-        <v>40663.58</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <f aca="false">SUM(F6:F7)</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="n">
-        <f aca="false">SUM(G6:G7)</f>
-        <v>178067.03</v>
-      </c>
-      <c r="H8" s="14" t="n">
-        <f aca="false">SUM(H6:H7)</f>
-        <v>91932.97</v>
-      </c>
-      <c r="I8" s="15" t="n">
-        <f aca="false">IF(B8=0,"",G8/B8)</f>
-        <v>0.659507518518519</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!F6:F8)</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!F9:F11)</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="10" t="n">
-        <f aca="false">SUM('Monthly Spend'!F12:F14)</f>
-        <v>229.56</v>
-      </c>
-      <c r="F10" s="9" t="n">
-        <f aca="false">SUM('Monthly Spend'!F15:F17)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <f aca="false">SUM(C10:F10)</f>
-        <v>229.56</v>
-      </c>
-      <c r="H10" s="9" t="str">
-        <f aca="false">IF(B10="","",B10-G10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="12" t="str">
-        <f aca="false">IF(B10="","",G10/B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="14" t="n">
-        <f aca="false">C8+C10</f>
-        <v>75432.1</v>
-      </c>
-      <c r="D11" s="14" t="n">
-        <f aca="false">D8+D10</f>
-        <v>61971.35</v>
-      </c>
-      <c r="E11" s="14" t="n">
-        <f aca="false">E8+E10</f>
-        <v>40893.14</v>
-      </c>
-      <c r="F11" s="14" t="n">
-        <f aca="false">F8+F10</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="14" t="n">
-        <f aca="false">G8+G10</f>
-        <v>178296.59</v>
-      </c>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="11" t="n">
-        <f aca="false">E11</f>
-        <v>40893.14</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="11" t="n">
-        <f aca="false">G11</f>
-        <v>178296.59</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="11" t="n">
-        <f aca="false">B8</f>
-        <v>270000</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="11" t="n">
-        <f aca="false">H8</f>
-        <v>91932.97</v>
-      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="12" t="n">
+        <f aca="false">H9</f>
+        <v>-12139.8288</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="20" t="n">
         <v>350000</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="11" t="n">
-        <f aca="false">B19-G8</f>
-        <v>171932.97</v>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="12" t="n">
+        <f aca="false">B20-G9</f>
+        <v>67860.1712</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
-        <v>26</v>
+      <c r="A22" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <f aca="false">'Monthly Spend'!D17</f>
+        <v>89717.93</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I6:I10">
+  <conditionalFormatting sqref="I7:I11">
     <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0.9</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H6:H10">
+  <conditionalFormatting sqref="H7:H11">
     <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
+    <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1200,347 +1228,302 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="19" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="A2" s="19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="6" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>37</v>
       </c>
+      <c r="B5" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>8092.51</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>9697.47</v>
+      </c>
+      <c r="E5" s="23"/>
+      <c r="F5" s="12" t="n">
+        <f aca="false">C5+(D5+E5)*Summary!$B$3</f>
+        <v>19341.5752</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>8092.51</v>
-      </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="9" t="str">
-        <f aca="false">IF(D6="","",D6*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="11" t="n">
-        <f aca="false">SUM(C6,E6,F6)</f>
-        <v>8092.51</v>
+      <c r="C6" s="9" t="n">
+        <v>28952.75</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>9917.15</v>
+      </c>
+      <c r="E6" s="23"/>
+      <c r="F6" s="12" t="n">
+        <f aca="false">C6+(D6+E6)*Summary!$B$3</f>
+        <v>40456.644</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>28952.75</v>
-      </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="9" t="str">
-        <f aca="false">IF(D7="","",D7*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="11" t="n">
-        <f aca="false">SUM(C7,E7,F7)</f>
-        <v>28952.75</v>
+      <c r="B7" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>38386.84</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>9048.23</v>
+      </c>
+      <c r="E7" s="23"/>
+      <c r="F7" s="12" t="n">
+        <f aca="false">C7+(D7+E7)*Summary!$B$3</f>
+        <v>48882.7868</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>38386.84</v>
-      </c>
-      <c r="D8" s="21"/>
-      <c r="E8" s="9" t="str">
-        <f aca="false">IF(D8="","",D8*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="11" t="n">
-        <f aca="false">SUM(C8,E8,F8)</f>
-        <v>38386.84</v>
+      <c r="B8" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>22241.56</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>8922.13</v>
+      </c>
+      <c r="E8" s="23"/>
+      <c r="F8" s="12" t="n">
+        <f aca="false">C8+(D8+E8)*Summary!$B$3</f>
+        <v>32591.2308</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>22241.56</v>
-      </c>
-      <c r="D9" s="21"/>
-      <c r="E9" s="9" t="str">
-        <f aca="false">IF(D9="","",D9*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="11" t="n">
-        <f aca="false">SUM(C9,E9,F9)</f>
-        <v>22241.56</v>
+      <c r="C9" s="9" t="n">
+        <v>22276.5</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>10793.26</v>
+      </c>
+      <c r="E9" s="23"/>
+      <c r="F9" s="12" t="n">
+        <f aca="false">C9+(D9+E9)*Summary!$B$3</f>
+        <v>34796.6816</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>22276.5</v>
-      </c>
-      <c r="D10" s="21"/>
-      <c r="E10" s="9" t="str">
-        <f aca="false">IF(D10="","",D10*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="11" t="n">
-        <f aca="false">SUM(C10,E10,F10)</f>
-        <v>22276.5</v>
+      <c r="B10" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>17453.29</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>12486.7</v>
+      </c>
+      <c r="E10" s="23"/>
+      <c r="F10" s="12" t="n">
+        <f aca="false">C10+(D10+E10)*Summary!$B$3</f>
+        <v>31937.862</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>17453.29</v>
-      </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="9" t="str">
-        <f aca="false">IF(D11="","",D11*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="11" t="n">
-        <f aca="false">SUM(C11,E11,F11)</f>
-        <v>17453.29</v>
+      <c r="B11" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>18956.66</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>11763.61</v>
+      </c>
+      <c r="E11" s="23"/>
+      <c r="F11" s="12" t="n">
+        <f aca="false">C11+(D11+E11)*Summary!$B$3</f>
+        <v>32602.4476</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>18956.66</v>
-      </c>
-      <c r="D12" s="21"/>
-      <c r="E12" s="9" t="str">
-        <f aca="false">IF(D12="","",D12*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="11" t="n">
-        <f aca="false">SUM(C12,E12,F12)</f>
-        <v>18956.66</v>
+      <c r="C12" s="9" t="n">
+        <v>10643.94</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>10956.93</v>
+      </c>
+      <c r="E12" s="23"/>
+      <c r="F12" s="12" t="n">
+        <f aca="false">C12+(D12+E12)*Summary!$B$3</f>
+        <v>23353.9788</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>10643.94</v>
-      </c>
-      <c r="D13" s="21"/>
-      <c r="E13" s="9" t="str">
-        <f aca="false">IF(D13="","",D13*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="11" t="n">
-        <f aca="false">SUM(C13,E13,F13)</f>
-        <v>10643.94</v>
+      <c r="B13" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>11062.98</v>
+      </c>
+      <c r="D13" s="23" t="n">
+        <v>6132.45</v>
+      </c>
+      <c r="E13" s="23" t="n">
+        <v>229.56</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <f aca="false">C13+(D13+E13)*Summary!$B$3</f>
+        <v>18442.9116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>11062.98</v>
-      </c>
-      <c r="D14" s="21"/>
-      <c r="E14" s="9" t="str">
-        <f aca="false">IF(D14="","",D14*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F14" s="8" t="n">
+      <c r="B14" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="12" t="n">
+        <f aca="false">C14+(D14+E14)*Summary!$B$3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="12" t="n">
+        <f aca="false">C15+(D15+E15)*Summary!$B$3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="9"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="12" t="n">
+        <f aca="false">C16+(D16+E16)*Summary!$B$3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="18"/>
+      <c r="C17" s="15" t="n">
+        <f aca="false">SUM(C5:C16)</f>
+        <v>178067.03</v>
+      </c>
+      <c r="D17" s="24" t="n">
+        <f aca="false">SUM(D5:D16)</f>
+        <v>89717.93</v>
+      </c>
+      <c r="E17" s="24" t="n">
+        <f aca="false">SUM(E5:E16)</f>
         <v>229.56</v>
       </c>
-      <c r="G14" s="11" t="n">
-        <f aca="false">SUM(C14,E14,F14)</f>
-        <v>11292.54</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="9" t="str">
-        <f aca="false">IF(D15="","",D15*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="11" t="n">
-        <f aca="false">SUM(C15,E15,F15)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B16" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="9" t="str">
-        <f aca="false">IF(D16="","",D16*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="11" t="n">
-        <f aca="false">SUM(C16,E16,F16)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="9" t="str">
-        <f aca="false">IF(D17="","",D17*$C$3)</f>
-        <v/>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="11" t="n">
-        <f aca="false">SUM(C17,E17,F17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+      <c r="F17" s="15" t="n">
+        <f aca="false">SUM(F5:F16)</f>
+        <v>282406.1184</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="14" t="n">
-        <f aca="false">SUM(C6:C17)</f>
-        <v>178067.03</v>
-      </c>
-      <c r="D18" s="22" t="n">
-        <f aca="false">SUM(D6:D17)</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="14" t="n">
-        <f aca="false">SUM(E6:E17)</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="14" t="n">
-        <f aca="false">SUM(F6:F17)</f>
-        <v>229.56</v>
-      </c>
-      <c r="G18" s="14" t="n">
-        <f aca="false">SUM(G6:G17)</f>
-        <v>178296.59</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="19" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="19" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="19" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1576,366 +1559,366 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="23" t="n">
+      <c r="A5" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="17" t="n">
         <v>17825.83</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="17" t="n">
         <v>10450.84</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="12" t="n">
         <f aca="false">B5+C5</f>
         <v>28276.67</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="17" t="n">
         <v>26630.37</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="13" t="n">
         <f aca="false">IF(E5&gt;0,D5/E5,"")</f>
         <v>1.06182039528553</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="23" t="n">
+      <c r="A6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="17" t="n">
         <v>8520.2</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="17" t="n">
         <v>6026.61</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="12" t="n">
         <f aca="false">B6+C6</f>
         <v>14546.81</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="17" t="n">
         <v>29658.15</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <f aca="false">IF(E6&gt;0,D6/E6,"")</f>
         <v>0.490482717229497</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B7" s="23" t="n">
+      <c r="A7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="17" t="n">
         <v>8991.05</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="17" t="n">
         <v>3029.5</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="12" t="n">
         <f aca="false">B7+C7</f>
         <v>12020.55</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="17" t="n">
         <v>22995.72</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <f aca="false">IF(E7&gt;0,D7/E7,"")</f>
         <v>0.52272988190846</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" s="23" t="n">
+      <c r="A8" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="17" t="n">
         <v>7474.3</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="17" t="n">
         <v>1468.47</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="12" t="n">
         <f aca="false">B8+C8</f>
         <v>8942.77</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="17" t="n">
         <v>13663.52</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="13" t="n">
         <f aca="false">IF(E8&gt;0,D8/E8,"")</f>
         <v>0.654499718959682</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B9" s="23" t="n">
+      <c r="A9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="17" t="n">
         <v>5738.34</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="17" t="n">
         <v>5775.01</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="12" t="n">
         <f aca="false">B9+C9</f>
         <v>11513.35</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="17" t="n">
         <v>22327.18</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="13" t="n">
         <f aca="false">IF(E9&gt;0,D9/E9,"")</f>
         <v>0.515665211638908</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B10" s="23" t="n">
+      <c r="A10" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="17" t="n">
         <v>5475.19</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="17" t="n">
         <v>5942.62</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <f aca="false">B10+C10</f>
         <v>11417.81</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="17" t="n">
         <v>21992</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <f aca="false">IF(E10&gt;0,D10/E10,"")</f>
         <v>0.519180156420517</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B11" s="23" t="n">
+      <c r="A11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="17" t="n">
         <v>4435.23</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="17" t="n">
         <v>1951.21</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <f aca="false">B11+C11</f>
         <v>6386.44</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="17" t="n">
         <v>15328.36</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">IF(E11&gt;0,D11/E11,"")</f>
         <v>0.416642093479015</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B12" s="23" t="n">
+      <c r="A12" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="17" t="n">
         <v>4722.59</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="17" t="n">
         <v>1754.38</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <f aca="false">B12+C12</f>
         <v>6476.97</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="17" t="n">
         <v>13663.52</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">IF(E12&gt;0,D12/E12,"")</f>
         <v>0.474033777533169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B13" s="23" t="n">
+      <c r="A13" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="17" t="n">
         <v>29802.24</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="17" t="n">
         <v>17655.01</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <f aca="false">B13+C13</f>
         <v>47457.25</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="17" t="n">
         <v>27967.45</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">IF(E13&gt;0,D13/E13,"")</f>
         <v>1.69687440220685</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="23" t="n">
+      <c r="A14" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="17" t="n">
         <v>14033.47</v>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="17" t="n">
         <v>4412.69</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="12" t="n">
         <f aca="false">B14+C14</f>
         <v>18446.16</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="17" t="n">
         <v>22327.06</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">IF(E14&gt;0,D14/E14,"")</f>
         <v>0.826179532818024</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" s="23" t="n">
+      <c r="A15" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="17" t="n">
         <v>13603.69</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="17" t="n">
         <v>4415.75</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="12" t="n">
         <f aca="false">B15+C15</f>
         <v>18019.44</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="17" t="n">
         <v>22327.06</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">IF(E15&gt;0,D15/E15,"")</f>
         <v>0.80706729860537</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B16" s="23" t="n">
+      <c r="A16" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="17" t="n">
         <v>12132.84</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="17" t="n">
         <v>2356.54</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="12" t="n">
         <f aca="false">B16+C16</f>
         <v>14489.38</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="17" t="n">
         <v>18329.47</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="13" t="n">
         <f aca="false">IF(E16&gt;0,D16/E16,"")</f>
         <v>0.790496397331729</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B17" s="23" t="n">
+      <c r="A17" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="17" t="n">
         <v>8893.59</v>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="17" t="n">
         <v>1522.89</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="12" t="n">
         <f aca="false">B17+C17</f>
         <v>10416.48</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="17" t="n">
         <v>9498.98</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="13" t="n">
         <f aca="false">IF(E17&gt;0,D17/E17,"")</f>
         <v>1.09658931801099</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="23" t="n">
+      <c r="A18" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="17" t="n">
         <v>25413.03</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="17" t="n">
         <v>16094.63</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="12" t="n">
         <f aca="false">B18+C18</f>
         <v>41507.66</v>
       </c>
-      <c r="E18" s="23" t="n">
+      <c r="E18" s="17" t="n">
         <v>27967.45</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="13" t="n">
         <f aca="false">IF(E18&gt;0,D18/E18,"")</f>
         <v>1.48414174334807</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19" s="14" t="n">
+      <c r="A19" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="15" t="n">
         <f aca="false">SUM(B5:B18)</f>
         <v>167061.59</v>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="15" t="n">
         <f aca="false">SUM(C5:C18)</f>
         <v>82856.15</v>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D19" s="15" t="n">
         <f aca="false">SUM(D5:D18)</f>
         <v>249917.74</v>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E19" s="15" t="n">
         <f aca="false">SUM(E5:E18)</f>
         <v>294676.29</v>
       </c>
-      <c r="F19" s="15" t="n">
+      <c r="F19" s="16" t="n">
         <f aca="false">IF(E19&gt;0,D19/E19,"")</f>
         <v>0.848109428824423</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>78</v>
+      <c r="A20" s="19" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1967,78 +1950,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="s">
-        <v>80</v>
+      <c r="A3" s="25" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>81</v>
+      <c r="A4" s="25" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
-        <v>82</v>
+      <c r="A5" s="25" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>83</v>
+      <c r="A6" s="25" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>84</v>
+      <c r="A7" s="25" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24"/>
+      <c r="A8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
-        <v>85</v>
+      <c r="A9" s="26" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24"/>
+      <c r="A10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>86</v>
+      <c r="A11" s="26" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>87</v>
+      <c r="A12" s="25" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
-        <v>88</v>
+      <c r="A13" s="25" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
-        <v>89</v>
+      <c r="A14" s="25" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="24" t="s">
-        <v>90</v>
+      <c r="A15" s="25" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24" t="s">
-        <v>91</v>
+      <c r="A16" s="25" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24" t="s">
-        <v>92</v>
+      <c r="A17" s="25" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Set Google Ads budget to EUR 90k in spend workbook
Google budget is an EUR input converted to USD with the Summary rate;
adds Google budget left in EUR to the key numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jw6zcgNAxCa88wNrGAsFKC
</commit_message>
<xml_diff>
--- a/PNP_Paid_Ads_Spend_2026.xlsx
+++ b/PNP_Paid_Ads_Spend_2026.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="97">
   <si>
     <t xml:space="preserve">Plug and Play – Paid Ads Spend 2026</t>
   </si>
@@ -35,6 +35,12 @@
   </si>
   <si>
     <t xml:space="preserve">≈ 2026 average so far. Replace with the rate Finance uses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Ads budget (EUR):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google's budget is set in euros; converted to USD below with the rate above.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Spend vs. budget by platform (all in USD)</t>
@@ -77,7 +83,7 @@
     <t xml:space="preserve">Google Ads</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Meta + Google ($270k budget)</t>
+    <t xml:space="preserve">Total Meta + Google</t>
   </si>
   <si>
     <t xml:space="preserve">ChatGPT Ads (separate budget)</t>
@@ -86,7 +92,7 @@
     <t xml:space="preserve">Grand total – all platforms</t>
   </si>
   <si>
-    <t xml:space="preserve">Google Ads and ChatGPT Ads are billed in EUR and converted at the rate in B3. ChatGPT Ads is paid outside the $270k budget.</t>
+    <t xml:space="preserve">Google Ads and ChatGPT Ads are billed in EUR and converted at the rate in B3. ChatGPT Ads is paid outside the Meta + Google budget.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Key numbers</t>
@@ -111,6 +117,9 @@
   </si>
   <si>
     <t xml:space="preserve">Google Ads spent so far, in EUR (as billed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Ads budget left, in EUR</t>
   </si>
   <si>
     <t xml:space="preserve">Red = 90% or more of the annual budget already spent, or over budget.</t>
@@ -270,7 +279,7 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Red = over its territory budget. These territory budgets add up to $294,676, not $270,000, and its totals don't match the platform exports (Meta $167,062 vs $178,067; Google 82,856 vs €89,718).</t>
+    <t xml:space="preserve">Red = over its territory budget. These territory budgets add up to $294,676, which doesn't match the platform budgets, and its totals don't match the platform exports (Meta $167,062 vs $178,067; Google 82,856 vs €89,718).</t>
   </si>
   <si>
     <t xml:space="preserve">How to update this sheet</t>
@@ -297,10 +306,10 @@
     <t xml:space="preserve">Assumptions</t>
   </si>
   <si>
-    <t xml:space="preserve">• 2026 budget: Meta $180,000 + Google $90,000 = $270,000 (USD). Stretch to $350,000 under discussion, not approved.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• ChatGPT Ads is paid outside the $270k budget.</t>
+    <t xml:space="preserve">• 2026 budget: Meta $180,000 (USD) + Google €90,000 (EUR). Shown in USD on the Summary. Stretch to $350,000 under discussion, not approved.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ChatGPT Ads is paid outside the Meta + Google budget.</t>
   </si>
   <si>
     <t xml:space="preserve">• Last quarter = Q3 2026 (July–September).</t>
@@ -323,9 +332,9 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mmm\ d&quot;, &quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
-    <numFmt numFmtId="167" formatCode="\$#,##0;&quot;-$&quot;#,##0;\-"/>
-    <numFmt numFmtId="168" formatCode="0%;\-0%;\-"/>
-    <numFmt numFmtId="169" formatCode="\€#,##0;&quot;-€&quot;#,##0;\-"/>
+    <numFmt numFmtId="167" formatCode="\€#,##0;&quot;-€&quot;#,##0;\-"/>
+    <numFmt numFmtId="168" formatCode="\$#,##0;&quot;-$&quot;#,##0;\-"/>
+    <numFmt numFmtId="169" formatCode="0%;\-0%;\-"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -382,6 +391,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="12"/>
       <color rgb="FF1F3864"/>
@@ -392,14 +409,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <color rgb="FF595959"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -507,7 +516,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -532,7 +541,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -544,15 +561,51 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -560,51 +613,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -915,286 +928,307 @@
         <v>3</v>
       </c>
     </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>90000</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>4</v>
+      <c r="A5" s="8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="7" t="s">
+      <c r="A6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="B6" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="C6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="D6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="E6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="F6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
+      <c r="H6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="9" t="n">
+      <c r="A7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="11" t="n">
         <v>180000</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!C5:C7)</f>
         <v>75432.1</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!C8:C10)</f>
         <v>61971.35</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="13" t="n">
         <f aca="false">SUM('Monthly Spend'!C11:C13)</f>
         <v>40663.58</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!C14:C16)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="14" t="n">
         <f aca="false">SUM(C7:F7)</f>
         <v>178067.03</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="12" t="n">
         <f aca="false">IF(B7="","",B7-G7)</f>
         <v>1932.96999999997</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="15" t="n">
         <f aca="false">IF(B7="","",G7/B7)</f>
         <v>0.989261277777778</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>90000</v>
-      </c>
-      <c r="C8" s="10" t="n">
+      <c r="A8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <f aca="false">B4*B3</f>
+        <v>104400</v>
+      </c>
+      <c r="C8" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!D5:D7)*Summary!$B$3</f>
         <v>33248.906</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!D8:D10)*Summary!$B$3</f>
         <v>37354.4244</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="13" t="n">
         <f aca="false">SUM('Monthly Spend'!D11:D13)*Summary!$B$3</f>
         <v>33469.4684</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!D14:D16)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="14" t="n">
         <f aca="false">SUM(C8:F8)</f>
         <v>104072.7988</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="12" t="n">
         <f aca="false">IF(B8="","",B8-G8)</f>
-        <v>-14072.7988</v>
-      </c>
-      <c r="I8" s="13" t="n">
+        <v>327.20120000001</v>
+      </c>
+      <c r="I8" s="15" t="n">
         <f aca="false">IF(B8="","",G8/B8)</f>
-        <v>1.15636443111111</v>
+        <v>0.996865888888889</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="15" t="n">
+      <c r="A9" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="18" t="n">
         <f aca="false">SUM(B7:B8)</f>
-        <v>270000</v>
-      </c>
-      <c r="C9" s="15" t="n">
+        <v>284400</v>
+      </c>
+      <c r="C9" s="18" t="n">
         <f aca="false">SUM(C7:C8)</f>
         <v>108681.006</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="18" t="n">
         <f aca="false">SUM(D7:D8)</f>
         <v>99325.7744</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="18" t="n">
         <f aca="false">SUM(E7:E8)</f>
         <v>74133.0484</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="18" t="n">
         <f aca="false">SUM(F7:F8)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="18" t="n">
         <f aca="false">SUM(G7:G8)</f>
         <v>282139.8288</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="18" t="n">
         <f aca="false">SUM(H7:H8)</f>
-        <v>-12139.8288</v>
-      </c>
-      <c r="I9" s="16" t="n">
+        <v>2260.17119999998</v>
+      </c>
+      <c r="I9" s="19" t="n">
         <f aca="false">IF(B9=0,"",G9/B9)</f>
-        <v>1.04496232888889</v>
+        <v>0.992052843881857</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="10" t="n">
+      <c r="A11" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="20"/>
+      <c r="C11" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!E5:E7)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!E8:E10)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">SUM('Monthly Spend'!E11:E13)*Summary!$B$3</f>
         <v>266.2896</v>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="12" t="n">
         <f aca="false">SUM('Monthly Spend'!E14:E16)*Summary!$B$3</f>
         <v>0</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="14" t="n">
         <f aca="false">SUM(C11:F11)</f>
         <v>266.2896</v>
       </c>
-      <c r="H11" s="10" t="str">
+      <c r="H11" s="12" t="str">
         <f aca="false">IF(B11="","",B11-G11)</f>
         <v/>
       </c>
-      <c r="I11" s="13" t="str">
+      <c r="I11" s="15" t="str">
         <f aca="false">IF(B11="","",G11/B11)</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="15" t="n">
+      <c r="A12" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="21"/>
+      <c r="C12" s="18" t="n">
         <f aca="false">C9+C11</f>
         <v>108681.006</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="18" t="n">
         <f aca="false">D9+D11</f>
         <v>99325.7744</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="18" t="n">
         <f aca="false">E9+E11</f>
         <v>74399.338</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="18" t="n">
         <f aca="false">F9+F11</f>
         <v>0</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="18" t="n">
         <f aca="false">G9+G11</f>
         <v>282406.1184</v>
       </c>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>19</v>
+      <c r="A13" s="7" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>20</v>
+      <c r="A15" s="8" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="12" t="n">
+      <c r="A16" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="14" t="n">
         <f aca="false">E12</f>
         <v>74399.338</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="12" t="n">
+      <c r="A17" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="14" t="n">
         <f aca="false">G12</f>
         <v>282406.1184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="12" t="n">
+      <c r="A18" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="14" t="n">
         <f aca="false">B9</f>
-        <v>270000</v>
+        <v>284400</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="12" t="n">
+      <c r="A19" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="14" t="n">
         <f aca="false">H9</f>
-        <v>-12139.8288</v>
+        <v>2260.17119999998</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="20" t="n">
+      <c r="A20" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="22" t="n">
         <v>350000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="12" t="n">
+      <c r="A21" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="14" t="n">
         <f aca="false">B20-G9</f>
         <v>67860.1712</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="21" t="n">
+      <c r="A22" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="23" t="n">
         <f aca="false">'Monthly Spend'!D17</f>
         <v>89717.93</v>
       </c>
     </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="23" t="n">
+        <f aca="false">B4-'Monthly Spend'!D17</f>
+        <v>282.070000000007</v>
+      </c>
+    </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
-        <v>28</v>
+      <c r="A24" s="7" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1239,292 +1273,292 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
-        <v>30</v>
+      <c r="A2" s="7" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="A4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="B4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="C4" s="9" t="s">
         <v>36</v>
       </c>
+      <c r="D4" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="9" t="n">
+      <c r="A5" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="11" t="n">
         <v>8092.51</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="6" t="n">
         <v>9697.47</v>
       </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="12" t="n">
+      <c r="E5" s="6"/>
+      <c r="F5" s="14" t="n">
         <f aca="false">C5+(D5+E5)*Summary!$B$3</f>
         <v>19341.5752</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="9" t="n">
+      <c r="A6" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="11" t="n">
         <v>28952.75</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="6" t="n">
         <v>9917.15</v>
       </c>
-      <c r="E6" s="23"/>
-      <c r="F6" s="12" t="n">
+      <c r="E6" s="6"/>
+      <c r="F6" s="14" t="n">
         <f aca="false">C6+(D6+E6)*Summary!$B$3</f>
         <v>40456.644</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="9" t="n">
+      <c r="A7" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="11" t="n">
         <v>38386.84</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="6" t="n">
         <v>9048.23</v>
       </c>
-      <c r="E7" s="23"/>
-      <c r="F7" s="12" t="n">
+      <c r="E7" s="6"/>
+      <c r="F7" s="14" t="n">
         <f aca="false">C7+(D7+E7)*Summary!$B$3</f>
         <v>48882.7868</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="9" t="n">
+      <c r="A8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="11" t="n">
         <v>22241.56</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="6" t="n">
         <v>8922.13</v>
       </c>
-      <c r="E8" s="23"/>
-      <c r="F8" s="12" t="n">
+      <c r="E8" s="6"/>
+      <c r="F8" s="14" t="n">
         <f aca="false">C8+(D8+E8)*Summary!$B$3</f>
         <v>32591.2308</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="9" t="n">
+      <c r="A9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="11" t="n">
         <v>22276.5</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="6" t="n">
         <v>10793.26</v>
       </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="12" t="n">
+      <c r="E9" s="6"/>
+      <c r="F9" s="14" t="n">
         <f aca="false">C9+(D9+E9)*Summary!$B$3</f>
         <v>34796.6816</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="9" t="n">
+      <c r="A10" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="11" t="n">
         <v>17453.29</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="6" t="n">
         <v>12486.7</v>
       </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="12" t="n">
+      <c r="E10" s="6"/>
+      <c r="F10" s="14" t="n">
         <f aca="false">C10+(D10+E10)*Summary!$B$3</f>
         <v>31937.862</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="9" t="n">
+      <c r="A11" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="11" t="n">
         <v>18956.66</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="6" t="n">
         <v>11763.61</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="12" t="n">
+      <c r="E11" s="6"/>
+      <c r="F11" s="14" t="n">
         <f aca="false">C11+(D11+E11)*Summary!$B$3</f>
         <v>32602.4476</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="9" t="n">
+      <c r="A12" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>10643.94</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="6" t="n">
         <v>10956.93</v>
       </c>
-      <c r="E12" s="23"/>
-      <c r="F12" s="12" t="n">
+      <c r="E12" s="6"/>
+      <c r="F12" s="14" t="n">
         <f aca="false">C12+(D12+E12)*Summary!$B$3</f>
         <v>23353.9788</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="9" t="n">
+      <c r="A13" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="11" t="n">
         <v>11062.98</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="6" t="n">
         <v>6132.45</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="6" t="n">
         <v>229.56</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="14" t="n">
         <f aca="false">C13+(D13+E13)*Summary!$B$3</f>
         <v>18442.9116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="12" t="n">
+      <c r="A14" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="11"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="14" t="n">
         <f aca="false">C14+(D14+E14)*Summary!$B$3</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="12" t="n">
+      <c r="A15" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="14" t="n">
         <f aca="false">C15+(D15+E15)*Summary!$B$3</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="12" t="n">
+      <c r="A16" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="14" t="n">
         <f aca="false">C16+(D16+E16)*Summary!$B$3</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="15" t="n">
+      <c r="A17" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="18" t="n">
         <f aca="false">SUM(C5:C16)</f>
         <v>178067.03</v>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="25" t="n">
         <f aca="false">SUM(D5:D16)</f>
         <v>89717.93</v>
       </c>
-      <c r="E17" s="24" t="n">
+      <c r="E17" s="25" t="n">
         <f aca="false">SUM(E5:E16)</f>
         <v>229.56</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="18" t="n">
         <f aca="false">SUM(F5:F16)</f>
         <v>282406.1184</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>54</v>
+      <c r="A19" s="7" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
-        <v>55</v>
+      <c r="A20" s="7" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
-        <v>56</v>
+      <c r="A21" s="7" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>57</v>
+      <c r="A22" s="7" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1555,370 +1589,370 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="7" t="s">
+      <c r="A4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>13</v>
+      <c r="B4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="17" t="n">
+      <c r="A5" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="20" t="n">
         <v>17825.83</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="20" t="n">
         <v>10450.84</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="14" t="n">
         <f aca="false">B5+C5</f>
         <v>28276.67</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="20" t="n">
         <v>26630.37</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="15" t="n">
         <f aca="false">IF(E5&gt;0,D5/E5,"")</f>
         <v>1.06182039528553</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="17" t="n">
+      <c r="A6" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="20" t="n">
         <v>8520.2</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="20" t="n">
         <v>6026.61</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <f aca="false">B6+C6</f>
         <v>14546.81</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="20" t="n">
         <v>29658.15</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="15" t="n">
         <f aca="false">IF(E6&gt;0,D6/E6,"")</f>
         <v>0.490482717229497</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="17" t="n">
+      <c r="A7" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="20" t="n">
         <v>8991.05</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="20" t="n">
         <v>3029.5</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="14" t="n">
         <f aca="false">B7+C7</f>
         <v>12020.55</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="20" t="n">
         <v>22995.72</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="15" t="n">
         <f aca="false">IF(E7&gt;0,D7/E7,"")</f>
         <v>0.52272988190846</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" s="17" t="n">
+      <c r="A8" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="20" t="n">
         <v>7474.3</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="20" t="n">
         <v>1468.47</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="14" t="n">
         <f aca="false">B8+C8</f>
         <v>8942.77</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="20" t="n">
         <v>13663.52</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="15" t="n">
         <f aca="false">IF(E8&gt;0,D8/E8,"")</f>
         <v>0.654499718959682</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="17" t="n">
+      <c r="A9" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="20" t="n">
         <v>5738.34</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="20" t="n">
         <v>5775.01</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="14" t="n">
         <f aca="false">B9+C9</f>
         <v>11513.35</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="20" t="n">
         <v>22327.18</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="15" t="n">
         <f aca="false">IF(E9&gt;0,D9/E9,"")</f>
         <v>0.515665211638908</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B10" s="17" t="n">
+      <c r="A10" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="20" t="n">
         <v>5475.19</v>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="20" t="n">
         <v>5942.62</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="14" t="n">
         <f aca="false">B10+C10</f>
         <v>11417.81</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="20" t="n">
         <v>21992</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="15" t="n">
         <f aca="false">IF(E10&gt;0,D10/E10,"")</f>
         <v>0.519180156420517</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" s="17" t="n">
+      <c r="A11" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="20" t="n">
         <v>4435.23</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="20" t="n">
         <v>1951.21</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">B11+C11</f>
         <v>6386.44</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="20" t="n">
         <v>15328.36</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="15" t="n">
         <f aca="false">IF(E11&gt;0,D11/E11,"")</f>
         <v>0.416642093479015</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="17" t="n">
+      <c r="A12" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="20" t="n">
         <v>4722.59</v>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="20" t="n">
         <v>1754.38</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">B12+C12</f>
         <v>6476.97</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="20" t="n">
         <v>13663.52</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="15" t="n">
         <f aca="false">IF(E12&gt;0,D12/E12,"")</f>
         <v>0.474033777533169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B13" s="17" t="n">
+      <c r="A13" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="20" t="n">
         <v>29802.24</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="20" t="n">
         <v>17655.01</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">B13+C13</f>
         <v>47457.25</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="20" t="n">
         <v>27967.45</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="15" t="n">
         <f aca="false">IF(E13&gt;0,D13/E13,"")</f>
         <v>1.69687440220685</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="17" t="n">
+      <c r="A14" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="20" t="n">
         <v>14033.47</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="20" t="n">
         <v>4412.69</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">B14+C14</f>
         <v>18446.16</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="20" t="n">
         <v>22327.06</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="15" t="n">
         <f aca="false">IF(E14&gt;0,D14/E14,"")</f>
         <v>0.826179532818024</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="17" t="n">
+      <c r="A15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="20" t="n">
         <v>13603.69</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="20" t="n">
         <v>4415.75</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="14" t="n">
         <f aca="false">B15+C15</f>
         <v>18019.44</v>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="20" t="n">
         <v>22327.06</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="15" t="n">
         <f aca="false">IF(E15&gt;0,D15/E15,"")</f>
         <v>0.80706729860537</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="B16" s="17" t="n">
+      <c r="A16" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="20" t="n">
         <v>12132.84</v>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="20" t="n">
         <v>2356.54</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="14" t="n">
         <f aca="false">B16+C16</f>
         <v>14489.38</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="20" t="n">
         <v>18329.47</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="15" t="n">
         <f aca="false">IF(E16&gt;0,D16/E16,"")</f>
         <v>0.790496397331729</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="17" t="n">
+      <c r="A17" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="20" t="n">
         <v>8893.59</v>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="20" t="n">
         <v>1522.89</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="14" t="n">
         <f aca="false">B17+C17</f>
         <v>10416.48</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="20" t="n">
         <v>9498.98</v>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="F17" s="15" t="n">
         <f aca="false">IF(E17&gt;0,D17/E17,"")</f>
         <v>1.09658931801099</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="B18" s="17" t="n">
+      <c r="A18" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="20" t="n">
         <v>25413.03</v>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="20" t="n">
         <v>16094.63</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="14" t="n">
         <f aca="false">B18+C18</f>
         <v>41507.66</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="20" t="n">
         <v>27967.45</v>
       </c>
-      <c r="F18" s="13" t="n">
+      <c r="F18" s="15" t="n">
         <f aca="false">IF(E18&gt;0,D18/E18,"")</f>
         <v>1.48414174334807</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B19" s="15" t="n">
+      <c r="A19" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="18" t="n">
         <f aca="false">SUM(B5:B18)</f>
         <v>167061.59</v>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="C19" s="18" t="n">
         <f aca="false">SUM(C5:C18)</f>
         <v>82856.15</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="D19" s="18" t="n">
         <f aca="false">SUM(D5:D18)</f>
         <v>249917.74</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="18" t="n">
         <f aca="false">SUM(E5:E18)</f>
         <v>294676.29</v>
       </c>
-      <c r="F19" s="16" t="n">
+      <c r="F19" s="19" t="n">
         <f aca="false">IF(E19&gt;0,D19/E19,"")</f>
         <v>0.848109428824423</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
-        <v>79</v>
+      <c r="A20" s="7" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1950,78 +1984,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="25" t="s">
-        <v>81</v>
+      <c r="A3" s="26" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="25" t="s">
-        <v>82</v>
+      <c r="A4" s="26" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
-        <v>83</v>
+      <c r="A5" s="26" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>84</v>
+      <c r="A6" s="26" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>85</v>
+      <c r="A7" s="26" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25"/>
+      <c r="A8" s="26"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
-        <v>86</v>
+      <c r="A9" s="27" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25"/>
+      <c r="A10" s="26"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
-        <v>87</v>
+      <c r="A11" s="27" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
-        <v>88</v>
+      <c r="A12" s="26" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
-        <v>89</v>
+      <c r="A13" s="26" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
-        <v>90</v>
+      <c r="A14" s="26" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>91</v>
+      <c r="A15" s="26" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
-        <v>92</v>
+      <c r="A16" s="26" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>93</v>
+      <c r="A17" s="26" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Report 2026 spend workbook in EUR
Budgets assumed in EUR (Meta 180k + Google 90k = 270k, stretch 350k TBC);
Meta USD spend converted to EUR with the Summary rate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jw6zcgNAxCa88wNrGAsFKC
</commit_message>
<xml_diff>
--- a/PNP_Paid_Ads_Spend_2026.xlsx
+++ b/PNP_Paid_Ads_Spend_2026.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="94">
   <si>
     <t xml:space="preserve">Plug and Play – Paid Ads Spend 2026</t>
   </si>
@@ -31,19 +31,13 @@
     <t xml:space="preserve">Data up to:</t>
   </si>
   <si>
-    <t xml:space="preserve">EUR → USD rate used:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈ 2026 average so far. Replace with the rate Finance uses.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google Ads budget (EUR):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google's budget is set in euros; converted to USD below with the rate above.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Spend vs. budget by platform (all in USD)</t>
+    <t xml:space="preserve">Exchange rate (1 EUR = ? USD):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used only to convert Meta (billed in USD) to EUR. ≈ 2026 average so far – replace with Finance's rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Spend vs. budget by platform (all in EUR)</t>
   </si>
   <si>
     <t xml:space="preserve">Platform</t>
@@ -83,7 +77,7 @@
     <t xml:space="preserve">Google Ads</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Meta + Google</t>
+    <t xml:space="preserve">Total Meta + Google (€270k budget)</t>
   </si>
   <si>
     <t xml:space="preserve">ChatGPT Ads (separate budget)</t>
@@ -92,7 +86,7 @@
     <t xml:space="preserve">Grand total – all platforms</t>
   </si>
   <si>
-    <t xml:space="preserve">Google Ads and ChatGPT Ads are billed in EUR and converted at the rate in B3. ChatGPT Ads is paid outside the Meta + Google budget.</t>
+    <t xml:space="preserve">Meta is billed in USD and converted to EUR at the rate in B3. ChatGPT Ads is paid outside the €270k budget.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Key numbers</t>
@@ -110,16 +104,13 @@
     <t xml:space="preserve">Meta + Google budget left for Oct–Dec</t>
   </si>
   <si>
-    <t xml:space="preserve">Possible stretch budget (not approved)</t>
+    <t xml:space="preserve">Possible stretch budget (to be confirmed)</t>
   </si>
   <si>
     <t xml:space="preserve">Budget left for Oct–Dec if we stretch</t>
   </si>
   <si>
-    <t xml:space="preserve">Google Ads spent so far, in EUR (as billed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google Ads budget left, in EUR</t>
+    <t xml:space="preserve">For reference: Meta spent so far in USD (as billed)</t>
   </si>
   <si>
     <t xml:space="preserve">Red = 90% or more of the annual budget already spent, or over budget.</t>
@@ -128,7 +119,7 @@
     <t xml:space="preserve">Monthly Spend 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Amounts in the currency each platform bills in. Yellow cells = type here. The Total column converts everything to USD using the rate on the Summary tab.</t>
+    <t xml:space="preserve">Amounts in the currency each platform bills in. Yellow cells = type here. The Total column converts everything to EUR using the rate on the Summary tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Month</t>
@@ -150,7 +141,7 @@
   </si>
   <si>
     <t xml:space="preserve">Total
-(USD)</t>
+(EUR)</t>
   </si>
   <si>
     <t xml:space="preserve">Jan 2026</t>
@@ -291,10 +282,10 @@
     <t xml:space="preserve">2. Type each month's amount into the yellow cells on the 'Monthly Spend' tab.</t>
   </si>
   <si>
-    <t xml:space="preserve">   • Meta → 'Meta (USD)'   • Google → 'Google Ads (EUR)'   • ChatGPT → 'ChatGPT Ads (EUR)'  – the sheet converts EUR to USD by itself</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Change 'Data up to' on the Summary tab (and the EUR → USD rate if Finance gives you a new one).</t>
+    <t xml:space="preserve">   • Meta → 'Meta (USD)'   • Google → 'Google Ads (EUR)'   • ChatGPT → 'ChatGPT Ads (EUR)'  – the sheet converts Meta's USD to EUR by itself</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Change 'Data up to' on the Summary tab (and the exchange rate if Finance gives you a new one).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Everything else (quarters, totals, budget left) updates by itself.</t>
@@ -306,16 +297,16 @@
     <t xml:space="preserve">Assumptions</t>
   </si>
   <si>
-    <t xml:space="preserve">• 2026 budget: Meta $180,000 (USD) + Google €90,000 (EUR). Shown in USD on the Summary. Stretch to $350,000 under discussion, not approved.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• ChatGPT Ads is paid outside the Meta + Google budget.</t>
+    <t xml:space="preserve">• 2026 budget assumed in EUR: Meta €180,000 + Google €90,000 = €270,000. A stretch to €350,000 is to be confirmed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ChatGPT Ads is paid outside the €270k budget.</t>
   </si>
   <si>
     <t xml:space="preserve">• Last quarter = Q3 2026 (July–September).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Meta is billed in USD. Google Ads and ChatGPT Ads are billed in EUR → converted at the rate on the Summary tab (B3).</t>
+    <t xml:space="preserve">• Google Ads and ChatGPT Ads are billed in EUR. Meta is billed in USD → converted to EUR at the rate on the Summary tab (B3).</t>
   </si>
   <si>
     <t xml:space="preserve">• Spend = 'Amount spent' (Meta) / 'Cost' (Google) as reported by the platform, before tax.</t>
@@ -333,8 +324,8 @@
     <numFmt numFmtId="165" formatCode="mmm\ d&quot;, &quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="\€#,##0;&quot;-€&quot;#,##0;\-"/>
-    <numFmt numFmtId="168" formatCode="\$#,##0;&quot;-$&quot;#,##0;\-"/>
-    <numFmt numFmtId="169" formatCode="0%;\-0%;\-"/>
+    <numFmt numFmtId="168" formatCode="0%;\-0%;\-"/>
+    <numFmt numFmtId="169" formatCode="\$#,##0;&quot;-$&quot;#,##0;\-"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -391,14 +382,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <color rgb="FF595959"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="12"/>
       <color rgb="FF1F3864"/>
@@ -409,6 +392,14 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -541,15 +532,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -561,63 +544,71 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -895,7 +886,7 @@
   <dimension ref="A1:I24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
@@ -928,307 +919,286 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="n">
+    </row>
+    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>180000</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!C5:C7)/Summary!$B$3</f>
+        <v>65027.6724137931</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!C8:C10)/Summary!$B$3</f>
+        <v>53423.5775862069</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <f aca="false">SUM('Monthly Spend'!C11:C13)/Summary!$B$3</f>
+        <v>35054.8103448276</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!C14:C16)/Summary!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <f aca="false">SUM(C7:F7)</f>
+        <v>153506.060344828</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <f aca="false">IF(B7="","",B7-G7)</f>
+        <v>26493.9396551724</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <f aca="false">IF(B7="","",G7/B7)</f>
+        <v>0.852811446360153</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="9" t="n">
         <v>90000</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="11" t="n">
-        <v>180000</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!C5:C7)</f>
-        <v>75432.1</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!C8:C10)</f>
-        <v>61971.35</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <f aca="false">SUM('Monthly Spend'!C11:C13)</f>
-        <v>40663.58</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!C14:C16)</f>
+      <c r="C8" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!D5:D7)</f>
+        <v>28662.85</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!D8:D10)</f>
+        <v>32202.09</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <f aca="false">SUM('Monthly Spend'!D11:D13)</f>
+        <v>28852.99</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!D14:D16)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="14" t="n">
-        <f aca="false">SUM(C7:F7)</f>
-        <v>178067.03</v>
-      </c>
-      <c r="H7" s="12" t="n">
-        <f aca="false">IF(B7="","",B7-G7)</f>
-        <v>1932.96999999997</v>
-      </c>
-      <c r="I7" s="15" t="n">
-        <f aca="false">IF(B7="","",G7/B7)</f>
-        <v>0.989261277777778</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="16" t="n">
-        <f aca="false">B4*B3</f>
-        <v>104400</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!D5:D7)*Summary!$B$3</f>
-        <v>33248.906</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!D8:D10)*Summary!$B$3</f>
-        <v>37354.4244</v>
-      </c>
-      <c r="E8" s="13" t="n">
-        <f aca="false">SUM('Monthly Spend'!D11:D13)*Summary!$B$3</f>
-        <v>33469.4684</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!D14:D16)*Summary!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="n">
+      <c r="G8" s="12" t="n">
         <f aca="false">SUM(C8:F8)</f>
-        <v>104072.7988</v>
-      </c>
-      <c r="H8" s="12" t="n">
+        <v>89717.93</v>
+      </c>
+      <c r="H8" s="10" t="n">
         <f aca="false">IF(B8="","",B8-G8)</f>
-        <v>327.20120000001</v>
-      </c>
-      <c r="I8" s="15" t="n">
+        <v>282.069999999992</v>
+      </c>
+      <c r="I8" s="13" t="n">
         <f aca="false">IF(B8="","",G8/B8)</f>
         <v>0.996865888888889</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="18" t="n">
+      <c r="A9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="15" t="n">
         <f aca="false">SUM(B7:B8)</f>
-        <v>284400</v>
-      </c>
-      <c r="C9" s="18" t="n">
+        <v>270000</v>
+      </c>
+      <c r="C9" s="15" t="n">
         <f aca="false">SUM(C7:C8)</f>
-        <v>108681.006</v>
-      </c>
-      <c r="D9" s="18" t="n">
+        <v>93690.5224137931</v>
+      </c>
+      <c r="D9" s="15" t="n">
         <f aca="false">SUM(D7:D8)</f>
-        <v>99325.7744</v>
-      </c>
-      <c r="E9" s="18" t="n">
+        <v>85625.6675862069</v>
+      </c>
+      <c r="E9" s="15" t="n">
         <f aca="false">SUM(E7:E8)</f>
-        <v>74133.0484</v>
-      </c>
-      <c r="F9" s="18" t="n">
+        <v>63907.8003448276</v>
+      </c>
+      <c r="F9" s="15" t="n">
         <f aca="false">SUM(F7:F8)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="15" t="n">
         <f aca="false">SUM(G7:G8)</f>
-        <v>282139.8288</v>
-      </c>
-      <c r="H9" s="18" t="n">
+        <v>243223.990344828</v>
+      </c>
+      <c r="H9" s="15" t="n">
         <f aca="false">SUM(H7:H8)</f>
-        <v>2260.17119999998</v>
-      </c>
-      <c r="I9" s="19" t="n">
+        <v>26776.0096551724</v>
+      </c>
+      <c r="I9" s="16" t="n">
         <f aca="false">IF(B9=0,"",G9/B9)</f>
-        <v>0.992052843881857</v>
+        <v>0.900829593869732</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!E5:E7)*Summary!$B$3</f>
+      <c r="A11" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="17"/>
+      <c r="C11" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!E5:E7)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!E8:E10)*Summary!$B$3</f>
+      <c r="D11" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!E8:E10)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
-        <f aca="false">SUM('Monthly Spend'!E11:E13)*Summary!$B$3</f>
-        <v>266.2896</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <f aca="false">SUM('Monthly Spend'!E14:E16)*Summary!$B$3</f>
+      <c r="E11" s="11" t="n">
+        <f aca="false">SUM('Monthly Spend'!E11:E13)</f>
+        <v>229.56</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <f aca="false">SUM('Monthly Spend'!E14:E16)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G11" s="12" t="n">
         <f aca="false">SUM(C11:F11)</f>
-        <v>266.2896</v>
-      </c>
-      <c r="H11" s="12" t="str">
+        <v>229.56</v>
+      </c>
+      <c r="H11" s="10" t="str">
         <f aca="false">IF(B11="","",B11-G11)</f>
         <v/>
       </c>
-      <c r="I11" s="15" t="str">
+      <c r="I11" s="13" t="str">
         <f aca="false">IF(B11="","",G11/B11)</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="18" t="n">
+      <c r="A12" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="15" t="n">
         <f aca="false">C9+C11</f>
-        <v>108681.006</v>
-      </c>
-      <c r="D12" s="18" t="n">
+        <v>93690.5224137931</v>
+      </c>
+      <c r="D12" s="15" t="n">
         <f aca="false">D9+D11</f>
-        <v>99325.7744</v>
-      </c>
-      <c r="E12" s="18" t="n">
+        <v>85625.6675862069</v>
+      </c>
+      <c r="E12" s="15" t="n">
         <f aca="false">E9+E11</f>
-        <v>74399.338</v>
-      </c>
-      <c r="F12" s="18" t="n">
+        <v>64137.3603448276</v>
+      </c>
+      <c r="F12" s="15" t="n">
         <f aca="false">F9+F11</f>
         <v>0</v>
       </c>
-      <c r="G12" s="18" t="n">
+      <c r="G12" s="15" t="n">
         <f aca="false">G9+G11</f>
-        <v>282406.1184</v>
-      </c>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
+        <v>243453.550344828</v>
+      </c>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
+      <c r="B16" s="12" t="n">
+        <f aca="false">E12</f>
+        <v>64137.3603448276</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="B17" s="12" t="n">
+        <f aca="false">G12</f>
+        <v>243453.550344828</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="14" t="n">
-        <f aca="false">E12</f>
-        <v>74399.338</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+      <c r="B18" s="12" t="n">
+        <f aca="false">B9</f>
+        <v>270000</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="14" t="n">
-        <f aca="false">G12</f>
-        <v>282406.1184</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+      <c r="B19" s="12" t="n">
+        <f aca="false">H9</f>
+        <v>26776.0096551724</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="14" t="n">
-        <f aca="false">B9</f>
-        <v>284400</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+      <c r="B20" s="20" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="14" t="n">
-        <f aca="false">H9</f>
-        <v>2260.17119999998</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+      <c r="B21" s="12" t="n">
+        <f aca="false">B20-G9</f>
+        <v>106776.009655172</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="22" t="n">
-        <v>350000</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
+      <c r="B22" s="21" t="n">
+        <f aca="false">'Monthly Spend'!C17</f>
+        <v>178067.03</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
         <v>28</v>
-      </c>
-      <c r="B21" s="14" t="n">
-        <f aca="false">B20-G9</f>
-        <v>67860.1712</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="23" t="n">
-        <f aca="false">'Monthly Spend'!D17</f>
-        <v>89717.93</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="23" t="n">
-        <f aca="false">B4-'Monthly Spend'!D17</f>
-        <v>282.070000000007</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1273,292 +1243,292 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+      <c r="D4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="E4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="F4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="9" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="B5" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="C5" s="23" t="n">
+        <v>8092.51</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>9697.47</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="12" t="n">
+        <f aca="false">C5/Summary!$B$3+D5+E5</f>
+        <v>16673.7717241379</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="B6" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>28952.75</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>9917.15</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="12" t="n">
+        <f aca="false">C6/Summary!$B$3+D6+E6</f>
+        <v>34876.4172413793</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B7" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>38386.84</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>9048.23</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="12" t="n">
+        <f aca="false">C7/Summary!$B$3+D7+E7</f>
+        <v>42140.3334482759</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="11" t="n">
-        <v>8092.51</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>9697.47</v>
-      </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="14" t="n">
-        <f aca="false">C5+(D5+E5)*Summary!$B$3</f>
-        <v>19341.5752</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="B8" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>28952.75</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>9917.15</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="14" t="n">
-        <f aca="false">C6+(D6+E6)*Summary!$B$3</f>
-        <v>40456.644</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="C8" s="23" t="n">
+        <v>22241.56</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>8922.13</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="F8" s="12" t="n">
+        <f aca="false">C8/Summary!$B$3+D8+E8</f>
+        <v>28095.8886206897</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="11" t="n">
-        <v>38386.84</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>9048.23</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="14" t="n">
-        <f aca="false">C7+(D7+E7)*Summary!$B$3</f>
-        <v>48882.7868</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="B9" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>22276.5</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>10793.26</v>
+      </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="12" t="n">
+        <f aca="false">C9/Summary!$B$3+D9+E9</f>
+        <v>29997.1393103448</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B10" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>17453.29</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>12486.7</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="12" t="n">
+        <f aca="false">C10/Summary!$B$3+D10+E10</f>
+        <v>27532.6396551724</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="11" t="n">
-        <v>22241.56</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>8922.13</v>
-      </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="14" t="n">
-        <f aca="false">C8+(D8+E8)*Summary!$B$3</f>
-        <v>32591.2308</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="B11" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>22276.5</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>10793.26</v>
-      </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="14" t="n">
-        <f aca="false">C9+(D9+E9)*Summary!$B$3</f>
-        <v>34796.6816</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="C11" s="23" t="n">
+        <v>18956.66</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>11763.61</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="12" t="n">
+        <f aca="false">C11/Summary!$B$3+D11+E11</f>
+        <v>28105.5582758621</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>17453.29</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>12486.7</v>
-      </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="14" t="n">
-        <f aca="false">C10+(D10+E10)*Summary!$B$3</f>
-        <v>31937.862</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="B12" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>10643.94</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>10956.93</v>
+      </c>
+      <c r="E12" s="9"/>
+      <c r="F12" s="12" t="n">
+        <f aca="false">C12/Summary!$B$3+D12+E12</f>
+        <v>20132.7403448276</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B13" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>11062.98</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>6132.45</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>229.56</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <f aca="false">C13/Summary!$B$3+D13+E13</f>
+        <v>15899.0617241379</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>18956.66</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>11763.61</v>
-      </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="14" t="n">
-        <f aca="false">C11+(D11+E11)*Summary!$B$3</f>
-        <v>32602.4476</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+      <c r="B14" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>10643.94</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>10956.93</v>
-      </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="14" t="n">
-        <f aca="false">C12+(D12+E12)*Summary!$B$3</f>
-        <v>23353.9788</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="C14" s="23"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="12" t="n">
+        <f aca="false">C14/Summary!$B$3+D14+E14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="11" t="n">
-        <v>11062.98</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>6132.45</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>229.56</v>
-      </c>
-      <c r="F13" s="14" t="n">
-        <f aca="false">C13+(D13+E13)*Summary!$B$3</f>
-        <v>18442.9116</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+      <c r="B15" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="23"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="12" t="n">
+        <f aca="false">C15/Summary!$B$3+D15+E15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B16" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="23"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="12" t="n">
+        <f aca="false">C16/Summary!$B$3+D16+E16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="14" t="n">
-        <f aca="false">C14+(D14+E14)*Summary!$B$3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="14" t="n">
-        <f aca="false">C15+(D15+E15)*Summary!$B$3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="14" t="n">
-        <f aca="false">C16+(D16+E16)*Summary!$B$3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="18" t="n">
+      <c r="B17" s="18"/>
+      <c r="C17" s="24" t="n">
         <f aca="false">SUM(C5:C16)</f>
         <v>178067.03</v>
       </c>
-      <c r="D17" s="25" t="n">
+      <c r="D17" s="15" t="n">
         <f aca="false">SUM(D5:D16)</f>
         <v>89717.93</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="15" t="n">
         <f aca="false">SUM(E5:E16)</f>
         <v>229.56</v>
       </c>
-      <c r="F17" s="18" t="n">
+      <c r="F17" s="15" t="n">
         <f aca="false">SUM(F5:F16)</f>
-        <v>282406.1184</v>
+        <v>243453.550344828</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1589,370 +1559,370 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+      <c r="E4" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="9" t="s">
+      <c r="F4" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="25" t="n">
         <v>17825.83</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="25" t="n">
         <v>10450.84</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="21" t="n">
         <f aca="false">B5+C5</f>
         <v>28276.67</v>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="25" t="n">
         <v>26630.37</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="13" t="n">
         <f aca="false">IF(E5&gt;0,D5/E5,"")</f>
         <v>1.06182039528553</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="20" t="n">
+      <c r="A6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="25" t="n">
         <v>8520.2</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="25" t="n">
         <v>6026.61</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="21" t="n">
         <f aca="false">B6+C6</f>
         <v>14546.81</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="25" t="n">
         <v>29658.15</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="13" t="n">
         <f aca="false">IF(E6&gt;0,D6/E6,"")</f>
         <v>0.490482717229497</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" s="20" t="n">
+      <c r="A7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="25" t="n">
         <v>8991.05</v>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="25" t="n">
         <v>3029.5</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="21" t="n">
         <f aca="false">B7+C7</f>
         <v>12020.55</v>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="25" t="n">
         <v>22995.72</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="13" t="n">
         <f aca="false">IF(E7&gt;0,D7/E7,"")</f>
         <v>0.52272988190846</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="20" t="n">
+      <c r="A8" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="25" t="n">
         <v>7474.3</v>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="25" t="n">
         <v>1468.47</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="21" t="n">
         <f aca="false">B8+C8</f>
         <v>8942.77</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="25" t="n">
         <v>13663.52</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="13" t="n">
         <f aca="false">IF(E8&gt;0,D8/E8,"")</f>
         <v>0.654499718959682</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="20" t="n">
+      <c r="A9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="25" t="n">
         <v>5738.34</v>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="25" t="n">
         <v>5775.01</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="21" t="n">
         <f aca="false">B9+C9</f>
         <v>11513.35</v>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="25" t="n">
         <v>22327.18</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="13" t="n">
         <f aca="false">IF(E9&gt;0,D9/E9,"")</f>
         <v>0.515665211638908</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="B10" s="20" t="n">
+      <c r="A10" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="25" t="n">
         <v>5475.19</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="25" t="n">
         <v>5942.62</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="21" t="n">
         <f aca="false">B10+C10</f>
         <v>11417.81</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="25" t="n">
         <v>21992</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="13" t="n">
         <f aca="false">IF(E10&gt;0,D10/E10,"")</f>
         <v>0.519180156420517</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B11" s="20" t="n">
+      <c r="A11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="25" t="n">
         <v>4435.23</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="25" t="n">
         <v>1951.21</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="21" t="n">
         <f aca="false">B11+C11</f>
         <v>6386.44</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="25" t="n">
         <v>15328.36</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">IF(E11&gt;0,D11/E11,"")</f>
         <v>0.416642093479015</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="20" t="n">
+      <c r="A12" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="25" t="n">
         <v>4722.59</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="25" t="n">
         <v>1754.38</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="21" t="n">
         <f aca="false">B12+C12</f>
         <v>6476.97</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="25" t="n">
         <v>13663.52</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">IF(E12&gt;0,D12/E12,"")</f>
         <v>0.474033777533169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="20" t="n">
+      <c r="A13" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="25" t="n">
         <v>29802.24</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="25" t="n">
         <v>17655.01</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="21" t="n">
         <f aca="false">B13+C13</f>
         <v>47457.25</v>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="25" t="n">
         <v>27967.45</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">IF(E13&gt;0,D13/E13,"")</f>
         <v>1.69687440220685</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="B14" s="20" t="n">
+      <c r="A14" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="25" t="n">
         <v>14033.47</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="25" t="n">
         <v>4412.69</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="21" t="n">
         <f aca="false">B14+C14</f>
         <v>18446.16</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="25" t="n">
         <v>22327.06</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">IF(E14&gt;0,D14/E14,"")</f>
         <v>0.826179532818024</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B15" s="20" t="n">
+      <c r="A15" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="25" t="n">
         <v>13603.69</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="25" t="n">
         <v>4415.75</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="21" t="n">
         <f aca="false">B15+C15</f>
         <v>18019.44</v>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="25" t="n">
         <v>22327.06</v>
       </c>
-      <c r="F15" s="15" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">IF(E15&gt;0,D15/E15,"")</f>
         <v>0.80706729860537</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B16" s="20" t="n">
+      <c r="A16" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="25" t="n">
         <v>12132.84</v>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="25" t="n">
         <v>2356.54</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="21" t="n">
         <f aca="false">B16+C16</f>
         <v>14489.38</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="25" t="n">
         <v>18329.47</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="13" t="n">
         <f aca="false">IF(E16&gt;0,D16/E16,"")</f>
         <v>0.790496397331729</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B17" s="20" t="n">
+      <c r="A17" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="25" t="n">
         <v>8893.59</v>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="25" t="n">
         <v>1522.89</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="21" t="n">
         <f aca="false">B17+C17</f>
         <v>10416.48</v>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="25" t="n">
         <v>9498.98</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="13" t="n">
         <f aca="false">IF(E17&gt;0,D17/E17,"")</f>
         <v>1.09658931801099</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="B18" s="20" t="n">
+      <c r="A18" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="25" t="n">
         <v>25413.03</v>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="25" t="n">
         <v>16094.63</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="21" t="n">
         <f aca="false">B18+C18</f>
         <v>41507.66</v>
       </c>
-      <c r="E18" s="20" t="n">
+      <c r="E18" s="25" t="n">
         <v>27967.45</v>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="13" t="n">
         <f aca="false">IF(E18&gt;0,D18/E18,"")</f>
         <v>1.48414174334807</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B19" s="18" t="n">
+      <c r="A19" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="24" t="n">
         <f aca="false">SUM(B5:B18)</f>
         <v>167061.59</v>
       </c>
-      <c r="C19" s="18" t="n">
+      <c r="C19" s="24" t="n">
         <f aca="false">SUM(C5:C18)</f>
         <v>82856.15</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="24" t="n">
         <f aca="false">SUM(D5:D18)</f>
         <v>249917.74</v>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E19" s="24" t="n">
         <f aca="false">SUM(E5:E18)</f>
         <v>294676.29</v>
       </c>
-      <c r="F19" s="19" t="n">
+      <c r="F19" s="16" t="n">
         <f aca="false">IF(E19&gt;0,D19/E19,"")</f>
         <v>0.848109428824423</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>82</v>
+      <c r="A20" s="19" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1984,32 +1954,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2017,7 +1987,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2025,37 +1995,37 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>